<commit_message>
Deploying to gh-pages from @ RIVO-Noord/zorgviewer-ig@7a35763162a90d10fed8d5cec9d6eb1c30eee46c 🚀
</commit_message>
<xml_diff>
--- a/StructureDefinition-extension-Meta.source.xlsx
+++ b/StructureDefinition-extension-Meta.source.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/R4/StructureDefinition/extension-Meta.source</t>
+    <t>http://hl7.org/fhir/4.0/StructureDefinition/extension-Meta.source</t>
   </si>
   <si>
     <t>Version</t>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-02-21T07:54:13+00:00</t>
+    <t>2024-02-21T07:57:06+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>